<commit_message>
README: refinement in the customization section.
</commit_message>
<xml_diff>
--- a/doc/Project-info-locations.xlsx
+++ b/doc/Project-info-locations.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Locations" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Applicability" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Notes" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Types" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Symbols" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="110">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -30,7 +32,7 @@
     <t xml:space="preserve">Location</t>
   </si>
   <si>
-    <t xml:space="preserve">::source</t>
+    <t xml:space="preserve">`::source`</t>
   </si>
   <si>
     <t xml:space="preserve">`::search-in`</t>
@@ -292,6 +294,66 @@
   </si>
   <si>
     <t xml:space="preserve">A leading `/` designates the root of the classpath which may make sense in some environments and classloaders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`::type`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`::source` must evaluate to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any map that contains an `:aliases` entry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A string representing the path to a `deps.edn` file</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A string representing the path to a `deps.edn` resource file</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Symbol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Triggered logic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`'current-basis`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`clojure.java.basis/current-basis`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`'initial-basis`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`clojure.java.basis/initial-basis`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`'project-deps`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`'file`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`clojure.java.io/file`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`'resource`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`clojure.java.io/resource`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`'resource-cl`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`clojure.java.io/resource` with classloader</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`'read-edn`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`clojure.java.io/reader` + `clojure.tools.deps.edn/read-edn`</t>
   </si>
 </sst>
 </file>
@@ -302,7 +364,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -342,6 +404,17 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -385,7 +458,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -452,6 +525,22 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1235,4 +1324,157 @@
     <oddFooter>&amp;CPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="62.05"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="18" customFormat="true" ht="17.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+    </row>
+    <row r="2" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="17.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>94</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="17" width="62.05"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" location="clojure.java.basis/current-basis" display="`clojure.java.basis/current-basis`"/>
+    <hyperlink ref="B3" r:id="rId2" location="clojure.java.basis/initial-basis" display="`clojure.java.basis/initial-basis`"/>
+    <hyperlink ref="B4" r:id="rId3" location="clojure.tools.deps.edn/project-deps" display="`clojure.tools.deps.edn/project-deps`"/>
+    <hyperlink ref="B5" r:id="rId4" display="`clojure.java.io/file`"/>
+    <hyperlink ref="B6" r:id="rId5" display="`clojure.java.io/resource`"/>
+    <hyperlink ref="B7" r:id="rId6" display="`clojure.java.io/resource` with classloader"/>
+    <hyperlink ref="B8" r:id="rId7" location="clojure.tools.deps.edn/project-deps" display="`clojure.java.io/reader` + `clojure.tools.deps.edn/read-edn`"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;A</oddHeader>
+    <oddFooter>&amp;CPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
README: minor edit in the symbol table
</commit_message>
<xml_diff>
--- a/doc/Project-info-locations.xlsx
+++ b/doc/Project-info-locations.xlsx
@@ -317,40 +317,40 @@
     <t xml:space="preserve">Triggered logic</t>
   </si>
   <si>
-    <t xml:space="preserve">`'current-basis`</t>
+    <t xml:space="preserve">`current-basis`</t>
   </si>
   <si>
     <t xml:space="preserve">`clojure.java.basis/current-basis`</t>
   </si>
   <si>
-    <t xml:space="preserve">`'initial-basis`</t>
+    <t xml:space="preserve">`initial-basis`</t>
   </si>
   <si>
     <t xml:space="preserve">`clojure.java.basis/initial-basis`</t>
   </si>
   <si>
-    <t xml:space="preserve">`'project-deps`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`'file`</t>
+    <t xml:space="preserve">`project-deps`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`file`</t>
   </si>
   <si>
     <t xml:space="preserve">`clojure.java.io/file`</t>
   </si>
   <si>
-    <t xml:space="preserve">`'resource`</t>
+    <t xml:space="preserve">`resource`</t>
   </si>
   <si>
     <t xml:space="preserve">`clojure.java.io/resource`</t>
   </si>
   <si>
-    <t xml:space="preserve">`'resource-cl`</t>
+    <t xml:space="preserve">`resource-cl`</t>
   </si>
   <si>
     <t xml:space="preserve">`clojure.java.io/resource` with classloader</t>
   </si>
   <si>
-    <t xml:space="preserve">`'read-edn`</t>
+    <t xml:space="preserve">`read-edn`</t>
   </si>
   <si>
     <t xml:space="preserve">`clojure.java.io/reader` + `clojure.tools.deps.edn/read-edn`</t>
@@ -1403,7 +1403,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>97</v>
       </c>
@@ -1411,7 +1411,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
         <v>99</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>101</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>102</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>106</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="17.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>108</v>
       </c>

</xml_diff>